<commit_message>
Updated example of MarketResult model
</commit_message>
<xml_diff>
--- a/Instance/MarketCongestion/MarketCongestionEntities/GenerationTemplate/Espheim-MarketResult_MCE.xlsx
+++ b/Instance/MarketCongestion/MarketCongestionEntities/GenerationTemplate/Espheim-MarketResult_MCE.xlsx
@@ -5,27 +5,29 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erelanoalgaba\OneDrive - ENTSO-E\Documenten\GitHub\relicapgrid\Instance\MarketCongestion\MarketCongestionEntities\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erelanoalgaba\OneDrive - ENTSO-E\Documenten\GitHub\relicapgrid\Instance\MarketCongestion\MarketCongestionEntities\GenerationTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C84001E-4A1C-4CE4-BD5A-02562098BD09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1950FDA-1316-4073-A69C-06EFDCB6812C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28860" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-7788" windowWidth="30936" windowHeight="16776" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="169" r:id="rId1"/>
     <sheet name="Dataset" sheetId="170" r:id="rId2"/>
     <sheet name="MarketVenue" sheetId="2" r:id="rId3"/>
-    <sheet name="MarketProductType" sheetId="3" r:id="rId4"/>
-    <sheet name="MarketVenueProduct" sheetId="4" r:id="rId5"/>
-    <sheet name="MarketInstrument" sheetId="5" r:id="rId6"/>
+    <sheet name="MarketVenueOperator" sheetId="171" r:id="rId4"/>
+    <sheet name="MarketParticipant" sheetId="172" r:id="rId5"/>
+    <sheet name="MarketProductType" sheetId="3" r:id="rId6"/>
+    <sheet name="MarketVenueProduct" sheetId="4" r:id="rId7"/>
+    <sheet name="MarketInstrument" sheetId="5" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="311">
   <si>
     <t>Namespace prefix</t>
   </si>
@@ -198,9 +200,6 @@
     <t>cim:IdentifiedObject.name</t>
   </si>
   <si>
-    <t>Float</t>
-  </si>
-  <si>
     <t>Enumeration</t>
   </si>
   <si>
@@ -468,9 +467,6 @@
     <t>VenueProduct – TTF Gas Spot</t>
   </si>
   <si>
-    <t>TTF Gas Spot</t>
-  </si>
-  <si>
     <t>e5b7bd1a-b696-4b0b-9b33-37a24c3c4e31</t>
   </si>
   <si>
@@ -519,9 +515,6 @@
     <t>VenueProduct – NO2 aFRR energy</t>
   </si>
   <si>
-    <t>NO2 aFRR Energy</t>
-  </si>
-  <si>
     <t>d0210f5e-3cd1-4d91-9f40-8f6a5ab04fa3</t>
   </si>
   <si>
@@ -531,9 +524,6 @@
     <t>nc:MarketMatchingMethodKind.evaluation</t>
   </si>
   <si>
-    <t>nc:MarketInstrument.observedProperty</t>
-  </si>
-  <si>
     <t>nc:MarketInstrument.temporalApplicability</t>
   </si>
   <si>
@@ -546,9 +536,6 @@
     <t>nc:MarketInstrument.value</t>
   </si>
   <si>
-    <t>nc:MarketInstrument.marketAreaName</t>
-  </si>
-  <si>
     <t>FWD_NORDIC_M01-26</t>
   </si>
   <si>
@@ -844,6 +831,140 @@
   </si>
   <si>
     <t>nc:MarketProductType.kind</t>
+  </si>
+  <si>
+    <t>nc:MarketVenueOperator</t>
+  </si>
+  <si>
+    <t>MarketVenueOperator</t>
+  </si>
+  <si>
+    <t>Nord Pool AS</t>
+  </si>
+  <si>
+    <t>European Energy Exchange AG</t>
+  </si>
+  <si>
+    <t>This is EEX as a company and as described in their website
+https://www.eex.com/en/</t>
+  </si>
+  <si>
+    <t>This is Nord Pool as a company and as described in their website
+https://www.nordpoolgroup.com/en/About-us/</t>
+  </si>
+  <si>
+    <t>Statnett SF</t>
+  </si>
+  <si>
+    <t>This is Statnett as a company and as described in their website
+https://www.statnett.no/en/about-statnett/contact-us/</t>
+  </si>
+  <si>
+    <t>5c716dd2-84c6-4149-af86-e91e03efed12</t>
+  </si>
+  <si>
+    <t>224ac108-2f11-49a2-bd72-4cd3fe164465</t>
+  </si>
+  <si>
+    <t>eea9fcb3-dc1b-4937-8fdb-732d03fd3adb</t>
+  </si>
+  <si>
+    <t>_5c716dd2-84c6-4149-af86-e91e03efed12</t>
+  </si>
+  <si>
+    <t>_224ac108-2f11-49a2-bd72-4cd3fe164465</t>
+  </si>
+  <si>
+    <t>_eea9fcb3-dc1b-4937-8fdb-732d03fd3adb</t>
+  </si>
+  <si>
+    <t>nc:MarketParticipant</t>
+  </si>
+  <si>
+    <t>MarketParticipant</t>
+  </si>
+  <si>
+    <t>Arcane Energy ApS</t>
+  </si>
+  <si>
+    <t>This is a market participant of Nord Pool described in their website
+https://www.nordpoolgroup.com/en/trading/join-our-markets/membership/</t>
+  </si>
+  <si>
+    <t>01 Futura Solar Logistica Global SL</t>
+  </si>
+  <si>
+    <t>This is a market participant of EEX described in their website
+https://www.eex.com/en/trading-resources/participants/list-of-trading-participants</t>
+  </si>
+  <si>
+    <t>65cb54e3-26e9-4706-ad1e-aeb39a7218d0</t>
+  </si>
+  <si>
+    <t>bd837e79-6911-49b1-9336-271f658afe31</t>
+  </si>
+  <si>
+    <t>_65cb54e3-26e9-4706-ad1e-aeb39a7218d0</t>
+  </si>
+  <si>
+    <t>_bd837e79-6911-49b1-9336-271f658afe31</t>
+  </si>
+  <si>
+    <t>nc:MarketParticipant.MarketVenue</t>
+  </si>
+  <si>
+    <t>nc:MarketVenue.MarketVenueOperator</t>
+  </si>
+  <si>
+    <t>nc:MarketVenueProduct.baseCurrency</t>
+  </si>
+  <si>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>It goes to MCS</t>
+  </si>
+  <si>
+    <t>nc:MarketVenueProduct.observedProperty</t>
+  </si>
+  <si>
+    <t>_86349d15-641c-40e7-a1e7-061b157e12f5</t>
+  </si>
+  <si>
+    <t>86349d15-641c-40e7-a1e7-061b157e12f5</t>
+  </si>
+  <si>
+    <t>807d6544-5e73-4353-8088-2d9fcc91404c</t>
+  </si>
+  <si>
+    <t>_807d6544-5e73-4353-8088-2d9fcc91404c</t>
+  </si>
+  <si>
+    <t>NO2 aFRR Energy (price regulation)</t>
+  </si>
+  <si>
+    <t>NO2 aFRR Energy (volume regulation)</t>
+  </si>
+  <si>
+    <t>TTF Gas Spot (price)</t>
+  </si>
+  <si>
+    <t>TTF Gas Spot (volume)</t>
+  </si>
+  <si>
+    <t>nc:MarketProductType.chargeKind</t>
+  </si>
+  <si>
+    <t>[nc:ChargeKind.tax; nc:ChargeKind.levy; nc:ChargeKind.tariff; nc:ChargeKind.fee; nc:ChargeKind.surcharge; nc:ChargeKind.subsidy; nc:ChargeKind.other]</t>
+  </si>
+  <si>
+    <t>nc:ChargeKind.tax</t>
+  </si>
+  <si>
+    <t>nc:ChargeKind.fee</t>
+  </si>
+  <si>
+    <t>nc:ChargeKind.other</t>
   </si>
 </sst>
 </file>
@@ -886,7 +1007,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -896,6 +1017,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="40"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -927,7 +1054,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -945,6 +1072,16 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1323,13 +1460,13 @@
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F2" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -1343,10 +1480,10 @@
         <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -1360,10 +1497,10 @@
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
@@ -1377,10 +1514,10 @@
         <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
@@ -1393,6 +1530,12 @@
       <c r="C6" t="s">
         <v>8</v>
       </c>
+      <c r="D6" t="s">
+        <v>268</v>
+      </c>
+      <c r="E6" t="s">
+        <v>269</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -1403,6 +1546,12 @@
       </c>
       <c r="C7" t="s">
         <v>8</v>
+      </c>
+      <c r="D7" t="s">
+        <v>282</v>
+      </c>
+      <c r="E7" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
@@ -1527,13 +1676,13 @@
         <v>37</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>38</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:36" ht="58" x14ac:dyDescent="0.35">
@@ -1541,109 +1690,109 @@
         <v>40</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="Q2" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="R2" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="S2" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="U2" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="Q2" s="1" t="s">
+      <c r="V2" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="R2" s="1" t="s">
+      <c r="W2" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="X2" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="Y2" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="U2" s="1" t="s">
+      <c r="Z2" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="V2" s="1" t="s">
+      <c r="AA2" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="AB2" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="X2" s="1" t="s">
+      <c r="AC2" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="Y2" s="1" t="s">
+      <c r="AD2" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="Z2" s="1" t="s">
+      <c r="AE2" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="AA2" s="1" t="s">
+      <c r="AF2" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="AB2" s="1" t="s">
+      <c r="AG2" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="AC2" s="1" t="s">
+      <c r="AH2" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="AD2" s="1" t="s">
+      <c r="AI2" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="AE2" s="1" t="s">
+      <c r="AJ2" s="1" t="s">
         <v>243</v>
-      </c>
-      <c r="AF2" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="AG2" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="AH2" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="AI2" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="AJ2" s="1" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="3" spans="1:36" ht="29" x14ac:dyDescent="0.35">
@@ -1690,7 +1839,7 @@
         <v>50</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="P3" s="1" t="s">
         <v>50</v>
@@ -1747,7 +1896,7 @@
         <v>41</v>
       </c>
       <c r="AH3" s="1" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="AI3" s="1" t="s">
         <v>50</v>
@@ -1764,7 +1913,7 @@
         <v>52</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>52</v>
@@ -1773,13 +1922,13 @@
         <v>47</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>47</v>
@@ -1788,22 +1937,22 @@
         <v>47</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L4" s="1" t="s">
         <v>47</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="Q4" s="1" t="s">
         <v>47</v>
@@ -1812,19 +1961,19 @@
         <v>52</v>
       </c>
       <c r="S4" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="T4" s="1" t="s">
         <v>52</v>
       </c>
       <c r="U4" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="V4" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="V4" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="W4" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="X4" s="1" t="s">
         <v>52</v>
@@ -1833,16 +1982,16 @@
         <v>47</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="AA4" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AB4" s="1" t="s">
         <v>47</v>
       </c>
       <c r="AC4" s="1" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="AD4" s="1" t="s">
         <v>47</v>
@@ -1851,19 +2000,19 @@
         <v>47</v>
       </c>
       <c r="AF4" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="AG4" s="1" t="s">
         <v>47</v>
       </c>
       <c r="AH4" s="1" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="AI4" s="1" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="AJ4" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.35">
@@ -1874,7 +2023,7 @@
         <v>48</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>48</v>
@@ -1892,7 +2041,7 @@
         <v>43</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>48</v>
@@ -1901,7 +2050,7 @@
         <v>48</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="M5" s="1" t="s">
         <v>48</v>
@@ -1919,7 +2068,7 @@
         <v>48</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="S5" s="1" t="s">
         <v>43</v>
@@ -1934,13 +2083,13 @@
         <v>48</v>
       </c>
       <c r="W5" s="1" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="X5" s="1" t="s">
         <v>43</v>
       </c>
       <c r="Y5" s="1" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="Z5" s="1" t="s">
         <v>48</v>
@@ -1958,10 +2107,10 @@
         <v>43</v>
       </c>
       <c r="AE5" s="1" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="AF5" s="1" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="AG5" s="1" t="s">
         <v>48</v>
@@ -2093,56 +2242,56 @@
     </row>
     <row r="8" spans="1:36" ht="116" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="F8" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="H8" s="6" t="s">
         <v>257</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>262</v>
       </c>
       <c r="I8" s="6"/>
       <c r="M8" s="6" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="N8" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="O8" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="P8" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="R8" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="S8" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="T8" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="X8" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="O8" s="7" t="s">
+      <c r="AC8" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="AD8" s="7" t="s">
         <v>264</v>
       </c>
-      <c r="P8" s="6" t="s">
+      <c r="AF8" s="7" t="s">
         <v>265</v>
       </c>
-      <c r="R8" s="6" t="s">
+      <c r="AI8" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="AJ8" s="7" t="s">
         <v>266</v>
-      </c>
-      <c r="S8" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="T8" s="6" t="s">
-        <v>260</v>
-      </c>
-      <c r="X8" s="6" t="s">
-        <v>267</v>
-      </c>
-      <c r="AC8" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="AD8" s="7" t="s">
-        <v>269</v>
-      </c>
-      <c r="AF8" s="7" t="s">
-        <v>270</v>
-      </c>
-      <c r="AI8" s="6" t="s">
-        <v>261</v>
-      </c>
-      <c r="AJ8" s="7" t="s">
-        <v>271</v>
       </c>
     </row>
   </sheetData>
@@ -2158,23 +2307,24 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="36.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="47.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="68" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="37.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="34.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.08984375" customWidth="1"/>
+    <col min="5" max="5" width="37.1796875" customWidth="1"/>
+    <col min="6" max="6" width="28.26953125" customWidth="1"/>
+    <col min="7" max="7" width="34.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>38</v>
@@ -2183,35 +2333,38 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>50</v>
+      <c r="C3" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>50</v>
@@ -2222,16 +2375,19 @@
       <c r="F3" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G3" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>52</v>
+      <c r="C4" s="3" t="s">
+        <v>47</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>52</v>
@@ -2242,35 +2398,41 @@
       <c r="F4" s="1" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G4" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="E5" s="1" t="s">
         <v>48</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G5" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="2" t="s">
         <v>46</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -2282,52 +2444,64 @@
       <c r="F6" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G6" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" t="s">
+        <v>276</v>
+      </c>
+      <c r="D8" t="s">
+        <v>71</v>
+      </c>
+      <c r="G8" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>76</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C8" t="s">
-        <v>72</v>
-      </c>
-      <c r="F8" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="B9" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C9" t="s">
+        <v>277</v>
+      </c>
+      <c r="D9" t="s">
         <v>77</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="G9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" t="s">
+        <v>278</v>
+      </c>
+      <c r="D10" t="s">
         <v>80</v>
       </c>
-      <c r="C9" t="s">
-        <v>78</v>
-      </c>
-      <c r="F9" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="G10" t="s">
         <v>82</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="C10" t="s">
-        <v>81</v>
-      </c>
-      <c r="F10" t="s">
-        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -2341,8 +2515,348 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{879F72E0-9E6C-4E52-B24F-69CBA8882E03}">
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="36.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="47.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>279</v>
+      </c>
+      <c r="B8" t="s">
+        <v>276</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="E8" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>280</v>
+      </c>
+      <c r="B9" t="s">
+        <v>277</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>272</v>
+      </c>
+      <c r="E9" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>281</v>
+      </c>
+      <c r="B10" t="s">
+        <v>278</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="E10" t="s">
+        <v>274</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49C89993-40B4-4FDB-B3A6-20BE01987D6F}">
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="39.6328125" customWidth="1"/>
+    <col min="2" max="2" width="41.54296875" customWidth="1"/>
+    <col min="3" max="3" width="35" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.7265625" customWidth="1"/>
+    <col min="5" max="6" width="28.7265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>290</v>
+      </c>
+      <c r="B8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" t="s">
+        <v>288</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="F8" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>291</v>
+      </c>
+      <c r="B9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" t="s">
+        <v>289</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="F9" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B10" s="4"/>
+      <c r="D10" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.81640625" bestFit="1" customWidth="1"/>
@@ -2350,22 +2864,23 @@
     <col min="3" max="3" width="57.26953125" customWidth="1"/>
     <col min="4" max="4" width="29.54296875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="41.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="32.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.90625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="34.90625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="45.453125" customWidth="1"/>
-    <col min="10" max="10" width="35" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="34.6328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="43.7265625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="22.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.36328125" customWidth="1"/>
+    <col min="7" max="7" width="32.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="33.26953125" customWidth="1"/>
+    <col min="9" max="9" width="34.90625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="45.453125" customWidth="1"/>
+    <col min="11" max="11" width="35" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="34.6328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="43.7265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="22.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>38</v>
@@ -2374,77 +2889,80 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="C2" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="H2" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="I2" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="H2" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>119</v>
-      </c>
       <c r="J2" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>62</v>
+        <v>57</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="G3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="I3" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>50</v>
+      <c r="J3" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="K3" s="1" t="s">
         <v>50</v>
@@ -2455,37 +2973,40 @@
       <c r="M3" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" ht="246.5" x14ac:dyDescent="0.35">
+      <c r="N3" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>52</v>
+      <c r="J4" s="3" t="s">
+        <v>119</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>52</v>
@@ -2496,8 +3017,11 @@
       <c r="M4" s="1" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N4" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>43</v>
       </c>
@@ -2525,20 +3049,23 @@
       <c r="I5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K5" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="K5" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="L5" s="1" t="s">
         <v>48</v>
       </c>
       <c r="M5" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N5" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>44</v>
       </c>
@@ -2578,157 +3105,172 @@
       <c r="M6" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N6" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D8" t="s">
+        <v>98</v>
+      </c>
+      <c r="E8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F8" t="s">
+        <v>308</v>
+      </c>
+      <c r="G8" t="s">
+        <v>99</v>
+      </c>
+      <c r="H8" t="s">
+        <v>100</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J8" s="5"/>
+      <c r="K8" t="s">
         <v>92</v>
       </c>
-      <c r="B8" t="s">
-        <v>97</v>
-      </c>
-      <c r="C8" t="s">
-        <v>98</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="M8" t="s">
+        <v>90</v>
+      </c>
+      <c r="N8" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>101</v>
+      </c>
+      <c r="B9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D9" t="s">
+        <v>106</v>
+      </c>
+      <c r="E9" t="s">
         <v>99</v>
       </c>
-      <c r="E8" t="s">
-        <v>100</v>
-      </c>
-      <c r="F8" t="s">
-        <v>100</v>
-      </c>
-      <c r="G8" t="s">
-        <v>101</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="I8" s="5"/>
-      <c r="J8" t="s">
-        <v>93</v>
-      </c>
-      <c r="L8" t="s">
-        <v>91</v>
-      </c>
-      <c r="M8" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>102</v>
-      </c>
-      <c r="B9" t="s">
-        <v>105</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="F9" t="s">
+        <v>308</v>
+      </c>
+      <c r="G9" t="s">
+        <v>99</v>
+      </c>
+      <c r="H9" t="s">
         <v>106</v>
       </c>
-      <c r="D9" t="s">
+      <c r="I9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="E9" t="s">
-        <v>100</v>
-      </c>
-      <c r="F9" t="s">
-        <v>100</v>
-      </c>
-      <c r="G9" t="s">
-        <v>107</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5" t="s">
-        <v>104</v>
-      </c>
+      <c r="L9" s="5"/>
       <c r="M9" s="5" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N9" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10" t="s">
+        <v>104</v>
+      </c>
+      <c r="C10" t="s">
+        <v>97</v>
+      </c>
+      <c r="D10" t="s">
+        <v>111</v>
+      </c>
+      <c r="E10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F10" t="s">
+        <v>309</v>
+      </c>
+      <c r="G10" t="s">
+        <v>99</v>
+      </c>
+      <c r="H10" t="s">
+        <v>106</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J10" s="5"/>
+      <c r="K10" t="s">
+        <v>110</v>
+      </c>
+      <c r="M10" t="s">
+        <v>108</v>
+      </c>
+      <c r="N10" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>114</v>
+      </c>
+      <c r="B11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C11" t="s">
+        <v>97</v>
+      </c>
+      <c r="D11" t="s">
+        <v>111</v>
+      </c>
+      <c r="E11" t="s">
+        <v>117</v>
+      </c>
+      <c r="F11" t="s">
+        <v>310</v>
+      </c>
+      <c r="G11" t="s">
+        <v>99</v>
+      </c>
+      <c r="H11" t="s">
+        <v>106</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="K11" t="s">
         <v>113</v>
       </c>
-      <c r="B10" t="s">
-        <v>105</v>
-      </c>
-      <c r="C10" t="s">
-        <v>98</v>
-      </c>
-      <c r="D10" t="s">
-        <v>112</v>
-      </c>
-      <c r="E10" t="s">
-        <v>107</v>
-      </c>
-      <c r="F10" t="s">
-        <v>100</v>
-      </c>
-      <c r="G10" t="s">
-        <v>107</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="I10" s="5"/>
-      <c r="J10" t="s">
-        <v>111</v>
-      </c>
-      <c r="L10" t="s">
-        <v>109</v>
-      </c>
-      <c r="M10" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+      <c r="M11" t="s">
         <v>115</v>
       </c>
-      <c r="B11" t="s">
-        <v>105</v>
-      </c>
-      <c r="C11" t="s">
-        <v>98</v>
-      </c>
-      <c r="D11" t="s">
-        <v>112</v>
-      </c>
-      <c r="E11" t="s">
-        <v>118</v>
-      </c>
-      <c r="F11" t="s">
-        <v>100</v>
-      </c>
-      <c r="G11" t="s">
-        <v>107</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="J11" t="s">
-        <v>114</v>
-      </c>
-      <c r="L11" t="s">
+      <c r="N11" t="s">
         <v>116</v>
-      </c>
-      <c r="M11" t="s">
-        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -2736,32 +3278,35 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="45.453125" customWidth="1"/>
     <col min="2" max="2" width="41.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.1796875" customWidth="1"/>
     <col min="4" max="4" width="34.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.90625" customWidth="1"/>
-    <col min="6" max="6" width="22.90625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="22.90625" customWidth="1"/>
-    <col min="9" max="9" width="33.1796875" customWidth="1"/>
-    <col min="10" max="10" width="36.6328125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="36.36328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.1796875" customWidth="1"/>
-    <col min="13" max="13" width="30" customWidth="1"/>
-    <col min="14" max="14" width="16.6328125" customWidth="1"/>
+    <col min="5" max="5" width="42.90625" customWidth="1"/>
+    <col min="6" max="6" width="36.90625" customWidth="1"/>
+    <col min="7" max="7" width="22.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="40.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="40.26953125" customWidth="1"/>
+    <col min="10" max="10" width="22.90625" customWidth="1"/>
+    <col min="11" max="11" width="33.1796875" customWidth="1"/>
+    <col min="12" max="12" width="36.6328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="36.36328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.1796875" customWidth="1"/>
+    <col min="15" max="15" width="30" customWidth="1"/>
+    <col min="16" max="16" width="31.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>67</v>
+      <c r="B1" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>38</v>
@@ -2770,51 +3315,57 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="I2" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="I2" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>41</v>
       </c>
@@ -2822,33 +3373,33 @@
         <v>41</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="G3" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>50</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>58</v>
+        <v>50</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>295</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="L3" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="L3" s="2" t="s">
         <v>50</v>
       </c>
       <c r="M3" s="1" t="s">
@@ -2857,8 +3408,14 @@
       <c r="N3" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" ht="174" x14ac:dyDescent="0.35">
+      <c r="O3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="174" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>42</v>
       </c>
@@ -2866,33 +3423,33 @@
         <v>47</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>137</v>
+      <c r="E4" s="1" t="s">
+        <v>173</v>
       </c>
       <c r="F4" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H4" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>142</v>
+      <c r="I4" s="2" t="s">
+        <v>160</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="L4" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="L4" s="2" t="s">
         <v>52</v>
       </c>
       <c r="M4" s="1" t="s">
@@ -2901,8 +3458,14 @@
       <c r="N4" s="1" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>43</v>
       </c>
@@ -2915,7 +3478,7 @@
       <c r="D5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="1" t="s">
         <v>48</v>
       </c>
       <c r="F5" s="2" t="s">
@@ -2933,20 +3496,26 @@
       <c r="J5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="K5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M5" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="L5" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="N5" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>44</v>
       </c>
@@ -2959,7 +3528,7 @@
       <c r="D6" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="1" t="s">
         <v>46</v>
       </c>
       <c r="F6" s="2" t="s">
@@ -2977,10 +3546,10 @@
       <c r="J6" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="K6" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="L6" s="1" t="s">
+      <c r="K6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="L6" s="2" t="s">
         <v>46</v>
       </c>
       <c r="M6" s="1" t="s">
@@ -2989,214 +3558,333 @@
       <c r="N6" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>131</v>
+      </c>
+      <c r="B8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C8" t="s">
+        <v>132</v>
+      </c>
+      <c r="D8" t="s">
+        <v>135</v>
+      </c>
+      <c r="E8" t="s">
+        <v>172</v>
+      </c>
+      <c r="F8" t="s">
+        <v>137</v>
+      </c>
+      <c r="G8" t="s">
+        <v>138</v>
+      </c>
+      <c r="H8" t="s">
+        <v>139</v>
+      </c>
+      <c r="I8" t="s">
+        <v>177</v>
+      </c>
+      <c r="J8" t="s">
+        <v>140</v>
+      </c>
+      <c r="K8" t="s">
+        <v>143</v>
+      </c>
+      <c r="L8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M8" t="s">
+        <v>130</v>
+      </c>
+      <c r="O8" t="s">
+        <v>128</v>
+      </c>
+      <c r="P8" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" t="s">
+        <v>148</v>
+      </c>
+      <c r="D9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E9" t="s">
+        <v>172</v>
+      </c>
+      <c r="F9" t="s">
+        <v>149</v>
+      </c>
+      <c r="G9" t="s">
+        <v>151</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="I9" t="s">
+        <v>177</v>
+      </c>
+      <c r="K9" t="s">
+        <v>142</v>
+      </c>
+      <c r="L9" t="s">
+        <v>107</v>
+      </c>
+      <c r="M9" t="s">
+        <v>146</v>
+      </c>
+      <c r="O9" t="s">
+        <v>145</v>
+      </c>
+      <c r="P9" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>298</v>
+      </c>
+      <c r="B10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" t="s">
+        <v>148</v>
+      </c>
+      <c r="D10" t="s">
+        <v>135</v>
+      </c>
+      <c r="E10" t="s">
+        <v>188</v>
+      </c>
+      <c r="F10" t="s">
+        <v>149</v>
+      </c>
+      <c r="G10" t="s">
+        <v>151</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="I10" t="s">
+        <v>177</v>
+      </c>
+      <c r="K10" t="s">
+        <v>142</v>
+      </c>
+      <c r="L10" t="s">
+        <v>107</v>
+      </c>
+      <c r="M10" t="s">
+        <v>299</v>
+      </c>
+      <c r="O10" t="s">
+        <v>145</v>
+      </c>
+      <c r="P10" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>155</v>
+      </c>
+      <c r="B11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" t="s">
         <v>132</v>
       </c>
-      <c r="B9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C9" t="s">
-        <v>133</v>
-      </c>
-      <c r="D9" t="s">
-        <v>136</v>
-      </c>
-      <c r="E9" t="s">
-        <v>138</v>
-      </c>
-      <c r="F9" t="s">
-        <v>139</v>
-      </c>
-      <c r="G9" t="s">
+      <c r="D11" t="s">
+        <v>135</v>
+      </c>
+      <c r="E11" t="s">
+        <v>172</v>
+      </c>
+      <c r="F11" t="s">
+        <v>157</v>
+      </c>
+      <c r="G11" t="s">
+        <v>158</v>
+      </c>
+      <c r="H11" t="s">
+        <v>159</v>
+      </c>
+      <c r="I11" t="s">
+        <v>177</v>
+      </c>
+      <c r="J11" t="s">
         <v>140</v>
       </c>
-      <c r="H9" t="s">
-        <v>141</v>
-      </c>
-      <c r="I9" t="s">
-        <v>144</v>
-      </c>
-      <c r="J9" t="s">
-        <v>93</v>
-      </c>
-      <c r="K9" t="s">
-        <v>131</v>
-      </c>
-      <c r="M9" t="s">
-        <v>129</v>
-      </c>
-      <c r="N9" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>158</v>
-      </c>
-      <c r="B10" t="s">
-        <v>78</v>
-      </c>
-      <c r="C10" t="s">
-        <v>150</v>
-      </c>
-      <c r="D10" t="s">
-        <v>136</v>
-      </c>
-      <c r="E10" t="s">
-        <v>151</v>
-      </c>
-      <c r="F10" t="s">
-        <v>153</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="I10" t="s">
-        <v>143</v>
-      </c>
-      <c r="J10" t="s">
-        <v>108</v>
-      </c>
-      <c r="K10" t="s">
-        <v>148</v>
-      </c>
-      <c r="M10" t="s">
-        <v>146</v>
-      </c>
-      <c r="N10" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>157</v>
-      </c>
-      <c r="B11" t="s">
-        <v>72</v>
-      </c>
-      <c r="C11" t="s">
-        <v>133</v>
-      </c>
-      <c r="D11" t="s">
-        <v>136</v>
-      </c>
-      <c r="E11" t="s">
-        <v>159</v>
-      </c>
-      <c r="F11" t="s">
-        <v>160</v>
-      </c>
-      <c r="G11" t="s">
-        <v>161</v>
-      </c>
-      <c r="H11" t="s">
-        <v>141</v>
-      </c>
-      <c r="I11" t="s">
-        <v>143</v>
-      </c>
-      <c r="J11" t="s">
-        <v>111</v>
-      </c>
       <c r="K11" t="s">
-        <v>156</v>
+        <v>142</v>
       </c>
       <c r="L11" t="s">
-        <v>161</v>
+        <v>110</v>
       </c>
       <c r="M11" t="s">
         <v>154</v>
       </c>
       <c r="N11" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+        <v>159</v>
+      </c>
+      <c r="O11" t="s">
+        <v>152</v>
+      </c>
+      <c r="P11" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C12" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="D12" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E12" t="s">
+        <v>200</v>
+      </c>
+      <c r="F12" t="s">
+        <v>157</v>
+      </c>
+      <c r="G12" t="s">
+        <v>158</v>
+      </c>
+      <c r="H12" t="s">
         <v>159</v>
       </c>
-      <c r="F12" t="s">
-        <v>160</v>
-      </c>
-      <c r="G12" t="s">
+      <c r="I12" t="s">
+        <v>177</v>
+      </c>
+      <c r="K12" t="s">
+        <v>142</v>
+      </c>
+      <c r="L12" t="s">
+        <v>113</v>
+      </c>
+      <c r="M12" t="s">
+        <v>162</v>
+      </c>
+      <c r="N12" t="s">
+        <v>159</v>
+      </c>
+      <c r="O12" t="s">
         <v>161</v>
       </c>
-      <c r="I12" t="s">
-        <v>143</v>
-      </c>
-      <c r="J12" t="s">
-        <v>114</v>
-      </c>
-      <c r="K12" t="s">
-        <v>165</v>
-      </c>
-      <c r="L12" t="s">
+      <c r="P12" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>301</v>
+      </c>
+      <c r="B13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" t="s">
+        <v>164</v>
+      </c>
+      <c r="D13" t="s">
+        <v>135</v>
+      </c>
+      <c r="E13" t="s">
+        <v>206</v>
+      </c>
+      <c r="F13" t="s">
+        <v>157</v>
+      </c>
+      <c r="G13" t="s">
+        <v>158</v>
+      </c>
+      <c r="H13" t="s">
+        <v>159</v>
+      </c>
+      <c r="I13" t="s">
+        <v>177</v>
+      </c>
+      <c r="K13" t="s">
+        <v>142</v>
+      </c>
+      <c r="L13" t="s">
+        <v>113</v>
+      </c>
+      <c r="M13" t="s">
+        <v>300</v>
+      </c>
+      <c r="N13" t="s">
+        <v>159</v>
+      </c>
+      <c r="O13" t="s">
         <v>161</v>
       </c>
-      <c r="M12" t="s">
-        <v>163</v>
-      </c>
-      <c r="N12" t="s">
-        <v>164</v>
+      <c r="P13" t="s">
+        <v>303</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G9" r:id="rId1" xr:uid="{0607B5F3-234E-4220-AB8B-D12D893EB80B}"/>
-    <hyperlink ref="G10" r:id="rId2" xr:uid="{9BF3749E-CA37-4D1D-895E-D453CD547D7C}"/>
+    <hyperlink ref="H8" r:id="rId1" xr:uid="{0607B5F3-234E-4220-AB8B-D12D893EB80B}"/>
+    <hyperlink ref="H9" r:id="rId2" xr:uid="{9BF3749E-CA37-4D1D-895E-D453CD547D7C}"/>
+    <hyperlink ref="H10" r:id="rId3" xr:uid="{A1B12320-F67E-45FA-8957-A26F12164FE2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.90625" customWidth="1"/>
-    <col min="2" max="2" width="36.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40.54296875" customWidth="1"/>
+    <col min="2" max="2" width="39.54296875" customWidth="1"/>
     <col min="3" max="3" width="53" customWidth="1"/>
     <col min="4" max="4" width="46.6328125" customWidth="1"/>
     <col min="5" max="5" width="36.6328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="29" customWidth="1"/>
+    <col min="7" max="7" width="29" customWidth="1"/>
+    <col min="8" max="8" width="41.1796875" customWidth="1"/>
+    <col min="9" max="9" width="29" customWidth="1"/>
     <col min="10" max="10" width="22.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="34.6328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="27.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="48.08984375" customWidth="1"/>
+    <col min="12" max="12" width="36.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>38</v>
@@ -3204,54 +3892,51 @@
       <c r="D1" s="1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+      <c r="F1" s="11" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="F2" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>171</v>
-      </c>
       <c r="G2" s="1" t="s">
-        <v>172</v>
+        <v>53</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>173</v>
+        <v>54</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="L2" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>58</v>
+      <c r="C3" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>50</v>
@@ -3259,14 +3944,14 @@
       <c r="E3" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="9" t="s">
         <v>50</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>50</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>50</v>
@@ -3274,37 +3959,31 @@
       <c r="J3" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="K3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="182" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:10" ht="182" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>178</v>
+      <c r="C4" s="1" t="s">
+        <v>60</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>47</v>
+      <c r="F4" s="9" t="s">
+        <v>62</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>52</v>
@@ -3312,14 +3991,8 @@
       <c r="J4" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="K4" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>43</v>
       </c>
@@ -3335,29 +4008,23 @@
       <c r="E5" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="9" t="s">
         <v>48</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>48</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K5" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>44</v>
       </c>
@@ -3373,7 +4040,7 @@
       <c r="E6" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="9" t="s">
         <v>46</v>
       </c>
       <c r="G6" s="1" t="s">
@@ -3388,220 +4055,179 @@
       <c r="J6" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K6" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="F7" s="10"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="B8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C8" t="s">
+        <v>174</v>
+      </c>
+      <c r="D8" t="s">
+        <v>176</v>
+      </c>
+      <c r="E8" t="s">
         <v>177</v>
       </c>
-      <c r="D8" t="s">
-        <v>179</v>
-      </c>
-      <c r="E8" t="s">
-        <v>181</v>
-      </c>
-      <c r="F8" t="s">
-        <v>182</v>
-      </c>
-      <c r="G8">
+      <c r="F8" s="10">
         <v>55.3</v>
       </c>
-      <c r="H8" t="s">
-        <v>139</v>
+      <c r="G8" t="s">
+        <v>170</v>
       </c>
       <c r="I8" t="s">
         <v>175</v>
       </c>
-      <c r="K8" t="s">
+      <c r="J8" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>182</v>
+      </c>
+      <c r="B9" t="s">
+        <v>146</v>
+      </c>
+      <c r="C9" t="s">
+        <v>183</v>
+      </c>
+      <c r="D9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E9" t="s">
+        <v>177</v>
+      </c>
+      <c r="F9" s="10">
+        <v>39.75</v>
+      </c>
+      <c r="G9" t="s">
+        <v>181</v>
+      </c>
+      <c r="I9" t="s">
+        <v>179</v>
+      </c>
+      <c r="J9" t="s">
         <v>180</v>
       </c>
-      <c r="L8" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>187</v>
       </c>
-      <c r="B9" t="s">
-        <v>148</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="B10" t="s">
+        <v>299</v>
+      </c>
+      <c r="C10" t="s">
+        <v>183</v>
+      </c>
+      <c r="D10" t="s">
+        <v>189</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="G10" t="s">
+        <v>186</v>
+      </c>
+      <c r="I10" t="s">
+        <v>184</v>
+      </c>
+      <c r="J10" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>194</v>
+      </c>
+      <c r="B11" t="s">
+        <v>154</v>
+      </c>
+      <c r="C11" t="s">
+        <v>195</v>
+      </c>
+      <c r="D11" t="s">
+        <v>176</v>
+      </c>
+      <c r="E11" t="s">
         <v>177</v>
       </c>
-      <c r="D9" t="s">
-        <v>188</v>
-      </c>
-      <c r="E9" t="s">
-        <v>181</v>
-      </c>
-      <c r="F9" t="s">
-        <v>182</v>
-      </c>
-      <c r="G9">
-        <v>39.75</v>
-      </c>
-      <c r="H9" t="s">
-        <v>153</v>
-      </c>
-      <c r="I9" t="s">
-        <v>186</v>
-      </c>
-      <c r="K9" t="s">
-        <v>184</v>
-      </c>
-      <c r="L9" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="F11" s="10">
+        <v>72.34</v>
+      </c>
+      <c r="G11" t="s">
+        <v>193</v>
+      </c>
+      <c r="I11" t="s">
+        <v>191</v>
+      </c>
+      <c r="J11" t="s">
         <v>192</v>
       </c>
-      <c r="B10" t="s">
-        <v>148</v>
-      </c>
-      <c r="C10" t="s">
-        <v>193</v>
-      </c>
-      <c r="D10" t="s">
-        <v>188</v>
-      </c>
-      <c r="E10" t="s">
-        <v>194</v>
-      </c>
-      <c r="G10" t="s">
-        <v>195</v>
-      </c>
-      <c r="H10" t="s">
-        <v>153</v>
-      </c>
-      <c r="I10" t="s">
-        <v>191</v>
-      </c>
-      <c r="K10" t="s">
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>199</v>
+      </c>
+      <c r="B12" t="s">
+        <v>162</v>
+      </c>
+      <c r="C12" t="s">
+        <v>201</v>
+      </c>
+      <c r="D12" t="s">
+        <v>176</v>
+      </c>
+      <c r="E12" t="s">
+        <v>177</v>
+      </c>
+      <c r="F12" s="10">
+        <v>145</v>
+      </c>
+      <c r="G12" t="s">
+        <v>198</v>
+      </c>
+      <c r="I12" t="s">
+        <v>196</v>
+      </c>
+      <c r="J12" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>205</v>
+      </c>
+      <c r="B13" t="s">
+        <v>300</v>
+      </c>
+      <c r="C13" t="s">
+        <v>201</v>
+      </c>
+      <c r="D13" t="s">
         <v>189</v>
       </c>
-      <c r="L10" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>199</v>
-      </c>
-      <c r="B11" t="s">
-        <v>156</v>
-      </c>
-      <c r="C11" t="s">
-        <v>177</v>
-      </c>
-      <c r="D11" t="s">
-        <v>200</v>
-      </c>
-      <c r="E11" t="s">
-        <v>181</v>
-      </c>
-      <c r="F11" t="s">
-        <v>182</v>
-      </c>
-      <c r="G11">
-        <v>72.34</v>
-      </c>
-      <c r="H11" t="s">
-        <v>160</v>
-      </c>
-      <c r="I11" t="s">
-        <v>198</v>
-      </c>
-      <c r="K11" t="s">
-        <v>196</v>
-      </c>
-      <c r="L11" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+      <c r="F13" s="10">
+        <v>7.5</v>
+      </c>
+      <c r="G13" t="s">
         <v>204</v>
       </c>
-      <c r="B12" t="s">
-        <v>165</v>
-      </c>
-      <c r="C12" t="s">
-        <v>205</v>
-      </c>
-      <c r="D12" t="s">
-        <v>206</v>
-      </c>
-      <c r="E12" t="s">
-        <v>181</v>
-      </c>
-      <c r="F12" t="s">
-        <v>182</v>
-      </c>
-      <c r="G12">
-        <v>145</v>
-      </c>
-      <c r="H12" t="s">
-        <v>160</v>
-      </c>
-      <c r="I12" t="s">
+      <c r="I13" t="s">
+        <v>202</v>
+      </c>
+      <c r="J13" t="s">
         <v>203</v>
-      </c>
-      <c r="K12" t="s">
-        <v>201</v>
-      </c>
-      <c r="L12" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>210</v>
-      </c>
-      <c r="B13" t="s">
-        <v>165</v>
-      </c>
-      <c r="C13" t="s">
-        <v>211</v>
-      </c>
-      <c r="D13" t="s">
-        <v>206</v>
-      </c>
-      <c r="E13" t="s">
-        <v>194</v>
-      </c>
-      <c r="G13">
-        <v>7.5</v>
-      </c>
-      <c r="H13" t="s">
-        <v>160</v>
-      </c>
-      <c r="I13" t="s">
-        <v>209</v>
-      </c>
-      <c r="K13" t="s">
-        <v>207</v>
-      </c>
-      <c r="L13" t="s">
-        <v>208</v>
       </c>
     </row>
   </sheetData>

</xml_diff>